<commit_message>
Update CYE passage planning — rebalance entries across Vendredi and Samedi
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/planning_passage_CYE.xlsx
+++ b/src/assets/planning_passage_CYE.xlsx
@@ -9,19 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="2364" windowHeight="0" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19368" windowHeight="9372" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Vendredi 17h" sheetId="1" r:id="rId1"/>
     <sheet name="Samedi 10h – Presentiel" sheetId="2" r:id="rId2"/>
     <sheet name="Samedi – Vue par Salle" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="229">
   <si>
     <t>N°</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Ahmed Dridi</t>
   </si>
   <si>
+    <t>Dialy-Help 🌐</t>
+  </si>
+  <si>
     <t>Zone B</t>
   </si>
   <si>
@@ -59,205 +62,325 @@
     <t>Salle CYE 1</t>
   </si>
   <si>
+    <t>JCI Sfax</t>
+  </si>
+  <si>
+    <t>Emna Moujehed</t>
+  </si>
+  <si>
+    <t>Zymotech 🌐</t>
+  </si>
+  <si>
+    <t>Zone E</t>
+  </si>
+  <si>
+    <t>Salle CYE 2</t>
+  </si>
+  <si>
+    <t>JCI Zarzis</t>
+  </si>
+  <si>
+    <t>Asma Basly</t>
+  </si>
+  <si>
+    <t>OORB - Open  Organic Robotics 🌐</t>
+  </si>
+  <si>
+    <t>17:10</t>
+  </si>
+  <si>
+    <t>JCI El Alia</t>
+  </si>
+  <si>
+    <t>Mootaz Hammami</t>
+  </si>
+  <si>
+    <t>EduHelper 🌐</t>
+  </si>
+  <si>
+    <t>JCI Sbikha</t>
+  </si>
+  <si>
+    <t>Hamden Nasri</t>
+  </si>
+  <si>
+    <t>Trip Hive technologies 🌐</t>
+  </si>
+  <si>
+    <t>Zone D</t>
+  </si>
+  <si>
+    <t>17:20</t>
+  </si>
+  <si>
+    <t>Ouardanine</t>
+  </si>
+  <si>
+    <t>Seddik Houimli</t>
+  </si>
+  <si>
+    <t>SupplyzPro 🌐</t>
+  </si>
+  <si>
+    <t>Zone C</t>
+  </si>
+  <si>
+    <t>Sousse</t>
+  </si>
+  <si>
+    <t>Ichrak Eddor Mnijli</t>
+  </si>
+  <si>
+    <t>HeroBee 🌐</t>
+  </si>
+  <si>
+    <t>17:30</t>
+  </si>
+  <si>
+    <t>JCI INSAT Tunis</t>
+  </si>
+  <si>
+    <t>Riadh Jouini</t>
+  </si>
+  <si>
+    <t>NartaQ 🌐</t>
+  </si>
+  <si>
+    <t>Zone A</t>
+  </si>
+  <si>
+    <t>JCI Monastir</t>
+  </si>
+  <si>
+    <t>Chouchane Amina</t>
+  </si>
+  <si>
+    <t>Karhabti.app 🌐</t>
+  </si>
+  <si>
+    <t>17:40</t>
+  </si>
+  <si>
+    <t>JCI Hammam Sousse</t>
+  </si>
+  <si>
+    <t>Moetaz Ben Charrada</t>
+  </si>
+  <si>
+    <t>HAIER HR 🌐</t>
+  </si>
+  <si>
+    <t>ANIS BELKAHLA</t>
+  </si>
+  <si>
+    <t>BARBARIJ 🌐</t>
+  </si>
+  <si>
+    <t>17:50</t>
+  </si>
+  <si>
+    <t>JCI Rafraf</t>
+  </si>
+  <si>
+    <t>Sarra Soussia</t>
+  </si>
+  <si>
+    <t>Save The Plate 🌐</t>
+  </si>
+  <si>
+    <t>JCI BENGUERDANE</t>
+  </si>
+  <si>
+    <t>FAKER CHOUIKHI</t>
+  </si>
+  <si>
+    <t>Watcher AI 🌐</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>JCI Carthage</t>
+  </si>
+  <si>
+    <t>Yassine Khelifi</t>
+  </si>
+  <si>
+    <t>BIOHEAT 🌐</t>
+  </si>
+  <si>
+    <t>JCI SBIKHA</t>
+  </si>
+  <si>
+    <t>Aziz Ghannem</t>
+  </si>
+  <si>
+    <t>AG Afro Solar / Olibueno 🌐</t>
+  </si>
+  <si>
+    <t>18:10</t>
+  </si>
+  <si>
+    <t>JCI Menzel Bourguiba</t>
+  </si>
+  <si>
+    <t>Firas Yousfi</t>
+  </si>
+  <si>
+    <t>CLICK AND WIN 🌐</t>
+  </si>
+  <si>
+    <t>Ghardimaou</t>
+  </si>
+  <si>
+    <t>Khouloud Mhamdi</t>
+  </si>
+  <si>
+    <t>ARKHOU DRONE 🌐</t>
+  </si>
+  <si>
+    <t>18:20</t>
+  </si>
+  <si>
+    <t>Ras Jebel</t>
+  </si>
+  <si>
+    <t>Mohamed Amine Amara</t>
+  </si>
+  <si>
+    <t>Edulylo 🌐</t>
+  </si>
+  <si>
+    <t>JCI Nabeul</t>
+  </si>
+  <si>
+    <t>Benameur Helmi</t>
+  </si>
+  <si>
+    <t>PEDAGO 🌐</t>
+  </si>
+  <si>
+    <t>18:30</t>
+  </si>
+  <si>
+    <t>JCI UJ Jendouba</t>
+  </si>
+  <si>
+    <t>Ameni</t>
+  </si>
+  <si>
+    <t>KIDDOS 🌐</t>
+  </si>
+  <si>
+    <t>JCI UJ JENDOUBA</t>
+  </si>
+  <si>
+    <t>Ala Eddine Dhaouafi</t>
+  </si>
+  <si>
+    <t>Melleya 🌐</t>
+  </si>
+  <si>
+    <t>18:40</t>
+  </si>
+  <si>
+    <t>INSAT Tunis</t>
+  </si>
+  <si>
+    <t>Oussama Ben Abdessalem</t>
+  </si>
+  <si>
+    <t>Carbon Jar 🌐</t>
+  </si>
+  <si>
+    <t>JCI Menzel Jemil</t>
+  </si>
+  <si>
+    <t>Fehmi Kharroubi</t>
+  </si>
+  <si>
+    <t>ExypnoTech Engineering Services</t>
+  </si>
+  <si>
+    <t>18:50</t>
+  </si>
+  <si>
+    <t>Jawher Makhlouf</t>
+  </si>
+  <si>
+    <t>NaturAdds</t>
+  </si>
+  <si>
+    <t>SAMEDI – À partir de 10h00  (Présentiel)</t>
+  </si>
+  <si>
+    <t>JCI El Jem</t>
+  </si>
+  <si>
+    <t>Nadia BOUZGARROU</t>
+  </si>
+  <si>
+    <t>ECUME LAB</t>
+  </si>
+  <si>
+    <t>10:00</t>
+  </si>
+  <si>
+    <t>Beni khaled</t>
+  </si>
+  <si>
+    <t>Meriem Louati</t>
+  </si>
+  <si>
+    <t>Art.tounsi</t>
+  </si>
+  <si>
+    <t>Bekalta</t>
+  </si>
+  <si>
+    <t>Mohsen Fennira</t>
+  </si>
+  <si>
+    <t>Dawwerbi</t>
+  </si>
+  <si>
+    <t>10:10</t>
+  </si>
+  <si>
+    <t>Ghada MEJRI</t>
+  </si>
+  <si>
+    <t>ECOMARC</t>
+  </si>
+  <si>
+    <t>L’OLM Diwan</t>
+  </si>
+  <si>
+    <t>Rafik Gharbi</t>
+  </si>
+  <si>
+    <t>Dootify</t>
+  </si>
+  <si>
+    <t>10:20</t>
+  </si>
+  <si>
+    <t>Hajeb Laayoun</t>
+  </si>
+  <si>
+    <t>Abdelhak Abbassi</t>
+  </si>
+  <si>
+    <t>AgroNoya</t>
+  </si>
+  <si>
     <t>JCI Bizerte</t>
   </si>
   <si>
     <t>Kawther MEKNI</t>
   </si>
   <si>
-    <t>Salle CYE 2</t>
-  </si>
-  <si>
-    <t>JCI Zarzis</t>
-  </si>
-  <si>
-    <t>Asma Basly</t>
-  </si>
-  <si>
-    <t>Zone E</t>
-  </si>
-  <si>
-    <t>JCI El Alia</t>
-  </si>
-  <si>
-    <t>Mootaz Hammami</t>
-  </si>
-  <si>
-    <t>JCI Sbikha</t>
-  </si>
-  <si>
-    <t>Hamden Nasri</t>
-  </si>
-  <si>
-    <t>Zone D</t>
-  </si>
-  <si>
-    <t>Ouardanine</t>
-  </si>
-  <si>
-    <t>Seddik Houimli</t>
-  </si>
-  <si>
-    <t>Zone C</t>
-  </si>
-  <si>
-    <t>Sousse</t>
-  </si>
-  <si>
-    <t>Ichrak Eddor Mnijli</t>
-  </si>
-  <si>
-    <t>JCI INSAT Tunis</t>
-  </si>
-  <si>
-    <t>Riadh Jouini</t>
-  </si>
-  <si>
-    <t>Zone A</t>
-  </si>
-  <si>
-    <t>JCI Monastir</t>
-  </si>
-  <si>
-    <t>Chouchane Amina</t>
-  </si>
-  <si>
-    <t>JCI Hammam Sousse</t>
-  </si>
-  <si>
-    <t>Moetaz Ben Charrada</t>
-  </si>
-  <si>
-    <t>ANIS BELKAHLA</t>
-  </si>
-  <si>
-    <t>JCI Rafraf</t>
-  </si>
-  <si>
-    <t>Sarra Soussia</t>
-  </si>
-  <si>
-    <t>JCI Carthage</t>
-  </si>
-  <si>
-    <t>Yassine Khelifi</t>
-  </si>
-  <si>
-    <t>JCI SBIKHA</t>
-  </si>
-  <si>
-    <t>Aziz Ghannem</t>
-  </si>
-  <si>
-    <t>JCI Menzel Bourguiba</t>
-  </si>
-  <si>
-    <t>Firas Yousfi</t>
-  </si>
-  <si>
-    <t>Ghardimaou</t>
-  </si>
-  <si>
-    <t>Khouloud Mhamdi</t>
-  </si>
-  <si>
-    <t>Ras Jebel</t>
-  </si>
-  <si>
-    <t>Mohamed Amine Amara</t>
-  </si>
-  <si>
-    <t>JCI UJ Jendouba</t>
-  </si>
-  <si>
-    <t>Ameni</t>
-  </si>
-  <si>
-    <t>JCI Menzel Jemil</t>
-  </si>
-  <si>
-    <t>Fehmi Kharroubi</t>
-  </si>
-  <si>
-    <t>ExypnoTech Engineering Services</t>
-  </si>
-  <si>
-    <t>Jawher Makhlouf</t>
-  </si>
-  <si>
-    <t>NaturAdds</t>
-  </si>
-  <si>
-    <t>SAMEDI – À partir de 10h00  (Présentiel)</t>
-  </si>
-  <si>
-    <t>JCI El Jem</t>
-  </si>
-  <si>
-    <t>Nadia BOUZGARROU</t>
-  </si>
-  <si>
-    <t>ECUME LAB</t>
-  </si>
-  <si>
-    <t>10:00</t>
-  </si>
-  <si>
-    <t>Beni khaled</t>
-  </si>
-  <si>
-    <t>Meriem Louati</t>
-  </si>
-  <si>
-    <t>Art.tounsi</t>
-  </si>
-  <si>
-    <t>Bekalta</t>
-  </si>
-  <si>
-    <t>Mohsen Fennira</t>
-  </si>
-  <si>
-    <t>Dawwerbi</t>
-  </si>
-  <si>
-    <t>10:10</t>
-  </si>
-  <si>
-    <t>JCI Sfax</t>
-  </si>
-  <si>
-    <t>Emna Moujehed</t>
-  </si>
-  <si>
-    <t>Zymotech</t>
-  </si>
-  <si>
-    <t>Ghada MEJRI</t>
-  </si>
-  <si>
-    <t>ECOMARC</t>
-  </si>
-  <si>
-    <t>10:20</t>
-  </si>
-  <si>
-    <t>L’OLM Diwan</t>
-  </si>
-  <si>
-    <t>Rafik Gharbi</t>
-  </si>
-  <si>
-    <t>Dootify</t>
-  </si>
-  <si>
-    <t>Hajeb Laayoun</t>
-  </si>
-  <si>
-    <t>Abdelhak Abbassi</t>
-  </si>
-  <si>
-    <t>AgroNoya</t>
+    <t>K Sustainova Consulting - Projet Lysitek 4 GPM</t>
   </si>
   <si>
     <t>10:30</t>
@@ -356,27 +479,18 @@
     <t>DDMLABS</t>
   </si>
   <si>
-    <t>JCI BENGUERDANE</t>
-  </si>
-  <si>
-    <t>FAKER CHOUIKHI</t>
-  </si>
-  <si>
-    <t>Watcher AI</t>
+    <t>jci zarzouna</t>
+  </si>
+  <si>
+    <t>Mustapha zoghlami</t>
+  </si>
+  <si>
+    <t>EL Makina digital</t>
   </si>
   <si>
     <t>11:20</t>
   </si>
   <si>
-    <t>jci zarzouna</t>
-  </si>
-  <si>
-    <t>Mustapha zoghlami</t>
-  </si>
-  <si>
-    <t>EL Makina digital</t>
-  </si>
-  <si>
     <t>JCI el manzah</t>
   </si>
   <si>
@@ -386,18 +500,18 @@
     <t>Omni Links TN</t>
   </si>
   <si>
+    <t>Gremda</t>
+  </si>
+  <si>
+    <t>Ahmed Walha</t>
+  </si>
+  <si>
+    <t>Dashmaster</t>
+  </si>
+  <si>
     <t>11:30</t>
   </si>
   <si>
-    <t>Gremda</t>
-  </si>
-  <si>
-    <t>Ahmed Walha</t>
-  </si>
-  <si>
-    <t>Dashmaster</t>
-  </si>
-  <si>
     <t>Ksar Saïd</t>
   </si>
   <si>
@@ -407,18 +521,18 @@
     <t>WIHELP</t>
   </si>
   <si>
+    <t>JCI TBS EL Mourouj</t>
+  </si>
+  <si>
+    <t>Khalil Jbeniani</t>
+  </si>
+  <si>
+    <t>Allcarta</t>
+  </si>
+  <si>
     <t>11:40</t>
   </si>
   <si>
-    <t>JCI TBS EL Mourouj</t>
-  </si>
-  <si>
-    <t>Khalil Jbeniani</t>
-  </si>
-  <si>
-    <t>Allcarta</t>
-  </si>
-  <si>
     <t>Bousalem</t>
   </si>
   <si>
@@ -428,15 +542,15 @@
     <t>The Denim Dilemma</t>
   </si>
   <si>
+    <t>Seif eddine BEN AMARA</t>
+  </si>
+  <si>
+    <t>Founder.tn</t>
+  </si>
+  <si>
     <t>11:50</t>
   </si>
   <si>
-    <t>Seif eddine BEN AMARA</t>
-  </si>
-  <si>
-    <t>Founder.tn</t>
-  </si>
-  <si>
     <t>JCI jardins El Mourouj</t>
   </si>
   <si>
@@ -446,21 +560,18 @@
     <t>MEPS (Methane Energy Production Solutions)</t>
   </si>
   <si>
+    <t>JCI Mornaguia</t>
+  </si>
+  <si>
+    <t>Aymen Masmoudi</t>
+  </si>
+  <si>
+    <t>LR MOVE</t>
+  </si>
+  <si>
     <t>12:00</t>
   </si>
   <si>
-    <t>JCI Mornaguia</t>
-  </si>
-  <si>
-    <t>Aymen Masmoudi</t>
-  </si>
-  <si>
-    <t>LR MOVE</t>
-  </si>
-  <si>
-    <t>JCI Feriana</t>
-  </si>
-  <si>
     <t>Dorra HERMASSI</t>
   </si>
   <si>
@@ -488,15 +599,6 @@
     <t>MIELVITA</t>
   </si>
   <si>
-    <t>JCI Nabeul</t>
-  </si>
-  <si>
-    <t>Benameur Helmi</t>
-  </si>
-  <si>
-    <t>PEDAGO</t>
-  </si>
-  <si>
     <t>Kelibia</t>
   </si>
   <si>
@@ -533,15 +635,6 @@
     <t>Ocotpus Agency</t>
   </si>
   <si>
-    <t>JCI UJ JENDOUBA</t>
-  </si>
-  <si>
-    <t>Ala Eddine Dhaouafi</t>
-  </si>
-  <si>
-    <t>Melleya</t>
-  </si>
-  <si>
     <t>medenine</t>
   </si>
   <si>
@@ -560,15 +653,6 @@
     <t>ROSNÉ</t>
   </si>
   <si>
-    <t>INSAT Tunis</t>
-  </si>
-  <si>
-    <t>Oussama Ben Abdessalem</t>
-  </si>
-  <si>
-    <t>Carbon Jar</t>
-  </si>
-  <si>
     <t>jci université jandouba</t>
   </si>
   <si>
@@ -614,70 +698,16 @@
     <t>Participant</t>
   </si>
   <si>
-    <t xml:space="preserve">Dialy-Help </t>
-  </si>
-  <si>
-    <t xml:space="preserve">K Sustainova Consulting - Projet Lysitek 4 GPM </t>
-  </si>
-  <si>
-    <t xml:space="preserve">OORB - Open  Organic Robotics </t>
-  </si>
-  <si>
-    <t xml:space="preserve">EduHelper </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trip Hive technologies </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SupplyzPro </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HeroBee </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NartaQ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karhabti.app </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HAIER HR </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BARBARIJ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Save The Plate </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIOHEAT </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AG Afro Solar / Olibueno </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLICK AND WIN </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARKHOU DRONE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edulylo </t>
-  </si>
-  <si>
-    <t xml:space="preserve">KIDDOS </t>
-  </si>
-  <si>
-    <t>JCI el jem</t>
-  </si>
-  <si>
-    <t>JCIEl Jem</t>
-  </si>
-  <si>
     <t>VENDREDI – À partir de 17h00  (En ligne )</t>
   </si>
   <si>
-    <t>JCI Gremda</t>
+    <t>JCI feriana</t>
+  </si>
+  <si>
+    <t>Jci Eljem</t>
+  </si>
+  <si>
+    <t>Ghada mejri</t>
   </si>
 </sst>
 </file>
@@ -726,7 +756,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -773,14 +803,8 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -803,50 +827,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-4.9989318521683403E-2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -928,6 +913,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -935,22 +923,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="20" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -960,27 +936,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1285,7 +1240,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1299,7 +1254,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -1342,16 +1297,16 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>197</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1359,22 +1314,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>198</v>
+        <v>15</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="32">
-        <v>0.71527777777777779</v>
+        <v>16</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1382,22 +1337,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="33">
-        <v>0.72222222222222221</v>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1405,22 +1360,22 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>200</v>
+        <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="32">
-        <v>0.72916666666666663</v>
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1428,22 +1383,22 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>201</v>
+        <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="33">
-        <v>0.73611111111111116</v>
+        <v>28</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1451,22 +1406,22 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>202</v>
+        <v>32</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="32">
-        <v>0.74305555555555547</v>
+        <v>33</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1474,22 +1429,22 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>203</v>
+        <v>36</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="33">
-        <v>0.75</v>
+        <v>33</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1497,22 +1452,22 @@
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>204</v>
+        <v>40</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="32">
-        <v>0.75694444444444453</v>
+        <v>41</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1520,22 +1475,22 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>205</v>
+        <v>44</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="32">
-        <v>0.76388888888888884</v>
+        <v>33</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1543,22 +1498,22 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="32">
-        <v>0.77083333333333337</v>
+      <c r="F12" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1566,22 +1521,22 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="32">
-        <v>0.77777777777777779</v>
+      <c r="F13" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1589,22 +1544,22 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>208</v>
+        <v>54</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="32">
-        <v>0.78472222222222221</v>
+        <v>10</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1612,22 +1567,22 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>209</v>
+        <v>57</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F15" s="32">
-        <v>0.79166666666666663</v>
+        <v>16</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1635,22 +1590,22 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="C16" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F16" s="32">
-        <v>0.79861111111111116</v>
+      <c r="F16" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1658,22 +1613,22 @@
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>211</v>
+        <v>64</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="32">
-        <v>0.80555555555555547</v>
+        <v>28</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1681,22 +1636,22 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>212</v>
+        <v>68</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="32">
-        <v>0.8125</v>
+        <v>10</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>65</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1704,22 +1659,22 @@
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>213</v>
+        <v>71</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="32">
-        <v>0.81944444444444453</v>
+        <v>10</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>72</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1727,41 +1682,161 @@
         <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>214</v>
+        <v>75</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="32">
-        <v>0.82638888888888884</v>
+        <v>10</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="44"/>
-      <c r="B21" s="42"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="44"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="44"/>
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="22" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="44"/>
-      <c r="B22" s="42"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="44"/>
+      <c r="A22" s="5">
+        <v>20</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="5">
+        <v>22</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="5">
+        <v>24</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1773,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1785,9 +1860,9 @@
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="27" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
@@ -1796,7 +1871,7 @@
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
     </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -1819,1045 +1894,915 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>2</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>63</v>
+        <v>104</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>4</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>67</v>
+        <v>226</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>68</v>
+        <v>183</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>69</v>
+        <v>184</v>
       </c>
       <c r="E6" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="33">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="K7" s="12"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+    </row>
+    <row r="8" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>6</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="E8" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>78</v>
+        <v>119</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
         <v>8</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>80</v>
+        <v>121</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>82</v>
+        <v>123</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>83</v>
+        <v>124</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>84</v>
+        <v>125</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <v>10</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>88</v>
+        <v>129</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
       <c r="E12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>90</v>
+        <v>131</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>91</v>
+        <v>132</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
         <v>12</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>94</v>
+        <v>135</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>95</v>
+        <v>136</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>98</v>
+        <v>139</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="12">
         <v>14</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>101</v>
+        <v>142</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>102</v>
+        <v>143</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>103</v>
+        <v>144</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>104</v>
+        <v>145</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="12">
         <v>16</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>109</v>
+        <v>150</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>17</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>111</v>
+        <v>152</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>112</v>
+        <v>153</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>113</v>
+        <v>154</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>114</v>
+        <v>155</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="12">
         <v>18</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>115</v>
+        <v>156</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>116</v>
+        <v>157</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>114</v>
+        <v>155</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>119</v>
+        <v>160</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12">
         <v>20</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>123</v>
+        <v>164</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="E22" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>127</v>
+        <v>168</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="12">
         <v>22</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="L24" s="12"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+    </row>
+    <row r="25" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12">
         <v>24</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>50</v>
+        <v>176</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>137</v>
+        <v>178</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>215</v>
+        <v>179</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>71</v>
+        <v>181</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>141</v>
+        <v>182</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="12">
         <v>26</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>142</v>
+        <v>97</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>141</v>
+        <v>33</v>
+      </c>
+      <c r="F28" s="33">
+        <v>0.5</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9">
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F29" s="34">
         <v>0.54861111111111105</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12">
         <v>28</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>148</v>
+        <v>18</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F30" s="35">
+        <v>16</v>
+      </c>
+      <c r="F30" s="33">
         <v>0.54861111111111105</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9">
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F31" s="34">
         <v>0.55555555555555558</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="12">
         <v>30</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>132</v>
+        <v>192</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>153</v>
+        <v>193</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>154</v>
+        <v>194</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F32" s="35">
+        <v>41</v>
+      </c>
+      <c r="F32" s="33">
         <v>0.55555555555555558</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9">
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>155</v>
+        <v>195</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>156</v>
+        <v>196</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F33" s="34">
         <v>0.5625</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12">
         <v>32</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>158</v>
+        <v>198</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F34" s="35">
+        <v>16</v>
+      </c>
+      <c r="F34" s="33">
         <v>0.5625</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9">
         <v>33</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>161</v>
+        <v>201</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>162</v>
+        <v>202</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>163</v>
+        <v>203</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F35" s="34">
         <v>0.56944444444444442</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="36" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="12">
         <v>34</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>164</v>
+        <v>204</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>165</v>
+        <v>205</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>166</v>
+        <v>206</v>
       </c>
       <c r="E36" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F36" s="33">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="G36" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F36" s="35">
-        <v>0.56944444444444442</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="37" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9">
         <v>35</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>167</v>
+        <v>207</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>168</v>
+        <v>208</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F37" s="34">
         <v>0.57638888888888895</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="12">
         <v>36</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F38" s="35">
+        <v>10</v>
+      </c>
+      <c r="F38" s="33">
         <v>0.57638888888888895</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>174</v>
+        <v>214</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>175</v>
+        <v>215</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F39" s="34">
         <v>0.58333333333333337</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q39" s="42"/>
-      <c r="R39" s="42"/>
-      <c r="S39" s="43"/>
-      <c r="T39" s="44"/>
-      <c r="U39" s="45"/>
-      <c r="V39" s="44"/>
-    </row>
-    <row r="40" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="12">
         <v>38</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>176</v>
+        <v>216</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>177</v>
+        <v>217</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>178</v>
+        <v>218</v>
       </c>
       <c r="E40" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="33">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="G40" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F40" s="35">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="G40" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="41" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9">
         <v>39</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F41" s="34">
         <v>0.59027777777777779</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12">
-        <v>40</v>
-      </c>
-      <c r="B42" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="E42" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" s="35">
-        <v>0.59027777777777779</v>
-      </c>
-      <c r="G42" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="9">
-        <v>41</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>187</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F43" s="34">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="44" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="12">
-        <v>42</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="D44" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F44" s="35">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="G44" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="9">
-        <v>43</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C45" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F45" s="34">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A46" s="41">
-        <v>44</v>
-      </c>
-      <c r="B46" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="C46" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="D46" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F46" s="35">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="G46" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A47" s="46">
-        <v>55</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="C47" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F47" s="34">
-        <v>0.61111111111111105</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2870,7 +2815,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -2889,39 +2834,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
-        <v>193</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
+      <c r="A1" s="32" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>194</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="H2" s="37" t="s">
-        <v>195</v>
-      </c>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="37"/>
-      <c r="M2" s="37"/>
+      <c r="A2" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="H2" s="29" t="s">
+        <v>223</v>
+      </c>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
     </row>
     <row r="3" spans="1:13" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
@@ -2931,7 +2872,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>196</v>
+        <v>224</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>3</v>
@@ -2942,22 +2883,22 @@
       <c r="F3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="36" t="s">
+      <c r="H3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="36" t="s">
-        <v>196</v>
-      </c>
-      <c r="K3" s="36" t="s">
+      <c r="J3" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="K3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="36" t="s">
+      <c r="L3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="36" t="s">
+      <c r="M3" s="8" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2966,37 +2907,37 @@
         <v>1</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="H4" s="19">
         <v>2</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="J4" s="20" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="L4" s="20" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3004,37 +2945,37 @@
         <v>3</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>63</v>
+        <v>104</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="H5" s="22">
         <v>4</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>67</v>
+        <v>226</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>68</v>
+        <v>183</v>
       </c>
       <c r="K5" s="24" t="s">
-        <v>69</v>
+        <v>184</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="M5" s="22" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3042,37 +2983,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="H6" s="19">
         <v>6</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>74</v>
+        <v>115</v>
       </c>
       <c r="K6" s="21" t="s">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="L6" s="20" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3080,37 +3021,37 @@
         <v>7</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>78</v>
+        <v>119</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
       <c r="H7" s="22">
         <v>8</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>80</v>
+        <v>121</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>82</v>
+        <v>123</v>
       </c>
       <c r="L7" s="23" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="M7" s="22" t="s">
-        <v>79</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3118,37 +3059,37 @@
         <v>9</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>83</v>
+        <v>124</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>84</v>
+        <v>125</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="H8" s="19">
         <v>10</v>
       </c>
       <c r="I8" s="20" t="s">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="J8" s="20" t="s">
-        <v>88</v>
+        <v>129</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
       <c r="L8" s="20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3156,37 +3097,37 @@
         <v>11</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>90</v>
+        <v>131</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>91</v>
+        <v>132</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
       <c r="H9" s="22">
         <v>12</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>94</v>
+        <v>135</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>95</v>
+        <v>136</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="L9" s="23" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="M9" s="22" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3194,37 +3135,37 @@
         <v>13</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>98</v>
+        <v>139</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="H10" s="19">
         <v>14</v>
       </c>
       <c r="I10" s="20" t="s">
-        <v>101</v>
+        <v>142</v>
       </c>
       <c r="J10" s="20" t="s">
-        <v>102</v>
+        <v>143</v>
       </c>
       <c r="K10" s="21" t="s">
-        <v>103</v>
+        <v>144</v>
       </c>
       <c r="L10" s="20" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3232,37 +3173,37 @@
         <v>15</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>104</v>
+        <v>145</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
       <c r="H11" s="22">
         <v>16</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>109</v>
+        <v>150</v>
       </c>
       <c r="K11" s="24" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="L11" s="23" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="M11" s="22" t="s">
-        <v>107</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3270,37 +3211,37 @@
         <v>17</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>111</v>
+        <v>152</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>112</v>
+        <v>153</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>113</v>
+        <v>154</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>114</v>
+        <v>155</v>
       </c>
       <c r="H12" s="19">
         <v>18</v>
       </c>
       <c r="I12" s="20" t="s">
-        <v>115</v>
+        <v>156</v>
       </c>
       <c r="J12" s="20" t="s">
-        <v>116</v>
+        <v>157</v>
       </c>
       <c r="K12" s="21" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="L12" s="20" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="M12" s="19" t="s">
-        <v>114</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3308,37 +3249,37 @@
         <v>19</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>119</v>
+        <v>160</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="H13" s="22">
         <v>20</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>123</v>
+        <v>164</v>
       </c>
       <c r="K13" s="24" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="M13" s="22" t="s">
-        <v>121</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3346,37 +3287,37 @@
         <v>21</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>126</v>
+        <v>167</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>127</v>
+        <v>168</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="H14" s="19">
         <v>22</v>
       </c>
       <c r="I14" s="20" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="K14" s="21" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="L14" s="20" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="M14" s="19" t="s">
-        <v>128</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3384,37 +3325,37 @@
         <v>23</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="H15" s="22">
         <v>24</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>50</v>
+        <v>176</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="K15" s="24" t="s">
-        <v>137</v>
+        <v>178</v>
       </c>
       <c r="L15" s="23" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3422,37 +3363,37 @@
         <v>25</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>216</v>
+        <v>179</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>71</v>
+        <v>181</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>141</v>
+        <v>182</v>
       </c>
       <c r="H16" s="19">
         <v>26</v>
       </c>
       <c r="I16" s="20" t="s">
-        <v>142</v>
+        <v>227</v>
       </c>
       <c r="J16" s="20" t="s">
-        <v>143</v>
+        <v>228</v>
       </c>
       <c r="K16" s="21" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="L16" s="20" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="M16" s="19" t="s">
-        <v>141</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3460,36 +3401,36 @@
         <v>27</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="D17" s="24" t="s">
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" s="38">
+        <v>10</v>
+      </c>
+      <c r="F17" s="35">
         <v>0.54861111111111105</v>
       </c>
       <c r="H17" s="22">
         <v>28</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>148</v>
+        <v>18</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="K17" s="24" t="s">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="L17" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="M17" s="38">
+        <v>16</v>
+      </c>
+      <c r="M17" s="35">
         <v>0.54861111111111105</v>
       </c>
     </row>
@@ -3498,36 +3439,36 @@
         <v>29</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="39">
+        <v>10</v>
+      </c>
+      <c r="F18" s="36">
         <v>0.55555555555555558</v>
       </c>
       <c r="H18" s="19">
         <v>30</v>
       </c>
       <c r="I18" s="20" t="s">
-        <v>132</v>
+        <v>192</v>
       </c>
       <c r="J18" s="20" t="s">
-        <v>153</v>
+        <v>193</v>
       </c>
       <c r="K18" s="21" t="s">
-        <v>154</v>
+        <v>194</v>
       </c>
       <c r="L18" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="M18" s="40">
+        <v>41</v>
+      </c>
+      <c r="M18" s="37">
         <v>0.55555555555555558</v>
       </c>
     </row>
@@ -3536,36 +3477,36 @@
         <v>31</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>155</v>
+        <v>195</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>156</v>
+        <v>196</v>
       </c>
       <c r="D19" s="24" t="s">
-        <v>157</v>
+        <v>197</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="F19" s="38">
+        <v>41</v>
+      </c>
+      <c r="F19" s="35">
         <v>0.5625</v>
       </c>
       <c r="H19" s="22">
         <v>32</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>158</v>
+        <v>198</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>159</v>
+        <v>199</v>
       </c>
       <c r="K19" s="24" t="s">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="L19" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="M19" s="38">
+        <v>16</v>
+      </c>
+      <c r="M19" s="35">
         <v>0.5625</v>
       </c>
     </row>
@@ -3574,36 +3515,36 @@
         <v>33</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>161</v>
+        <v>201</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>162</v>
+        <v>202</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>163</v>
+        <v>203</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F20" s="39">
+        <v>16</v>
+      </c>
+      <c r="F20" s="36">
         <v>0.56944444444444442</v>
       </c>
       <c r="H20" s="19">
         <v>34</v>
       </c>
       <c r="I20" s="20" t="s">
-        <v>164</v>
+        <v>204</v>
       </c>
       <c r="J20" s="20" t="s">
-        <v>165</v>
+        <v>205</v>
       </c>
       <c r="K20" s="21" t="s">
-        <v>166</v>
+        <v>206</v>
       </c>
       <c r="L20" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="M20" s="40">
+        <v>16</v>
+      </c>
+      <c r="M20" s="37">
         <v>0.56944444444444442</v>
       </c>
     </row>
@@ -3612,36 +3553,36 @@
         <v>35</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>167</v>
+        <v>207</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>168</v>
+        <v>208</v>
       </c>
       <c r="D21" s="24" t="s">
-        <v>169</v>
+        <v>209</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="38">
+        <v>16</v>
+      </c>
+      <c r="F21" s="35">
         <v>0.57638888888888895</v>
       </c>
       <c r="H21" s="22">
         <v>36</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>171</v>
+        <v>211</v>
       </c>
       <c r="K21" s="24" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="L21" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="M21" s="38">
+        <v>10</v>
+      </c>
+      <c r="M21" s="35">
         <v>0.57638888888888895</v>
       </c>
     </row>
@@ -3650,36 +3591,36 @@
         <v>37</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>173</v>
+        <v>213</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>174</v>
+        <v>214</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>175</v>
+        <v>215</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="39">
+        <v>41</v>
+      </c>
+      <c r="F22" s="36">
         <v>0.58333333333333337</v>
       </c>
       <c r="H22" s="19">
         <v>38</v>
       </c>
       <c r="I22" s="20" t="s">
-        <v>176</v>
+        <v>216</v>
       </c>
       <c r="J22" s="20" t="s">
-        <v>177</v>
+        <v>217</v>
       </c>
       <c r="K22" s="21" t="s">
-        <v>178</v>
+        <v>218</v>
       </c>
       <c r="L22" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="M22" s="40">
+        <v>10</v>
+      </c>
+      <c r="M22" s="37">
         <v>0.58333333333333337</v>
       </c>
     </row>
@@ -3688,141 +3629,26 @@
         <v>39</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="D23" s="24" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23" s="38">
+        <v>16</v>
+      </c>
+      <c r="F23" s="35">
         <v>0.59027777777777779</v>
-      </c>
-      <c r="H23" s="22">
-        <v>40</v>
-      </c>
-      <c r="I23" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="J23" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="K23" s="24" t="s">
-        <v>184</v>
-      </c>
-      <c r="L23" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="M23" s="38">
-        <v>0.59027777777777779</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="16">
-        <v>41</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="E24" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F24" s="39">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="H24" s="19">
-        <v>42</v>
-      </c>
-      <c r="I24" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="J24" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="K24" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="L24" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="M24" s="40">
-        <v>0.59722222222222221</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="22">
-        <v>43</v>
-      </c>
-      <c r="B25" s="42" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="E25" s="44" t="s">
-        <v>9</v>
-      </c>
-      <c r="F25" s="45">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="G25" s="44"/>
-      <c r="H25" s="47">
-        <v>44</v>
-      </c>
-      <c r="I25" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="J25" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="K25" s="24" t="s">
-        <v>192</v>
-      </c>
-      <c r="L25" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="M25" s="38">
-        <v>0.60416666666666663</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="16">
-        <v>41</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="E26" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="39">
-        <v>0.61111111111111105</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="H2:K2"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>